<commit_message>
Product sync logs added
</commit_message>
<xml_diff>
--- a/airtable_json_uploader/json_files/Airtable - 7 Colors.xlsx
+++ b/airtable_json_uploader/json_files/Airtable - 7 Colors.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="72">
   <si>
     <t>Product Code</t>
   </si>
@@ -130,35 +130,7 @@
     <t>{"Power": "7W", "Light Color": "Warm White", "Voltage": "12V/24V", "Current Type": "AC/DC", "IP Rating": "IP67", "Finish": "Black", "SKU": "GL001"}</t>
   </si>
   <si>
-    <t>{
-"Options": {
-"Power": [
-{"name": "7W", "id": "101"}
-],
-"Light Color": [
-{"name": "Warm White", "id": "102"}
-],
-"Voltage": [
-{"name": "12V/24V", "id": "103"}
-],
-"Current Type": [
-{"name": "AC/DC", "id": "104"}
-],
-"IP Rating": [
-{"name": "IP67", "id": "105"}
-],
-"Finish": [
-{"name": "Black", "id": "106"}
-]
-},
-"Constraints": {},
-"sku_mappings": [
-{
-"sku": "GL001",
-"combination": ["101", "102", "103", "104", "105", "106"]
-}
-]
-}</t>
+    <t>{"Options": {"Power": [{"name": "7W", "id": "101"}], "Light Color": [{"name": "Warm White", "id": "102"}], "Voltage": [{"name": "12V/24V", "id": "103"}], "Current Type": [{"name": "AC/DC", "id": "104"}], "IP Rating": [{"name": "IP67", "id": "105"}], "Finish": [{"name": "Black", "id": "106"}]}, "Constraints": {}, "sku_mappings": [{"sku": "GL001", "combination": ["101", "102", "103", "104", "105", "106"]}]}</t>
   </si>
   <si>
     <t>CHINA - 7 Colors Co Ltd</t>
@@ -224,13 +196,16 @@
     <t>7W | 3000K | 12V | IP68</t>
   </si>
   <si>
-    <t>Power|CCT|Voltage|IP Rating</t>
+    <t>Power|Color Temperature|Voltage|IP Rating</t>
   </si>
   <si>
-    <t>{"Power": "7W", "CCT": "3000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL001"}</t>
+    <t>{"Power": "7W", "Color Temperature": "3000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL001"}</t>
   </si>
   <si>
-    <t>{"Options": {"Power": [{"name": "7W", "id": "101"}], "CCT": [{"name": "3000K", "id": "102"}], "Voltage": [{"name": "12V", "id": "103"}], "IP Rating": [{"name": "IP68", "id": "104"}]}, "Constraints": {}, "sku_mappings": [{"sku": "PL001", "combination": ["101", "102", "103", "104"]}]}</t>
+    <t>{"Power": "7W", "Color Temperature": ["3000K", "6000K"], "Voltage": "12V", "IP Rating": "IP68", "SKU": ["PL001", "PL002"]}</t>
+  </si>
+  <si>
+    <t>{"Options": {"Power": [{"name": "7W", "id": "101"}], "Color Temperature": [{"name": "3000K", "id": "102"}, {"name": "6000K", "id": "103"}], "Voltage": [{"name": "12V", "id": "104"}], "IP Rating": [{"name": "IP68", "id": "105"}]}, "Constraints": {}, "sku_mappings": [{"sku": "PL001", "combination": ["101", "102", "104", "105"]}, {"sku": "PL002", "combination": ["101", "103", "104", "105"]}]}</t>
   </si>
   <si>
     <t>SC-G101A</t>
@@ -245,16 +220,16 @@
     <t>PL002</t>
   </si>
   <si>
-    <t>Transform your pool into a breathtaking oasis. Elevate your outdoor space with a sophisticated glow that brings enchanting elegance and serene luxury to every evening.</t>
-  </si>
-  <si>
     <t>7W | 6000K | 12V | IP68</t>
   </si>
   <si>
-    <t>{"Power": "7W", "CCT": "6000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL002"}</t>
-  </si>
-  <si>
-    <t>{"Options": {"Power": [{"name": "7W", "id": "101"}], "CCT": [{"name": "6000K", "id": "102"}], "Voltage": [{"name": "12V", "id": "103"}], "IP Rating": [{"name": "IP68", "id": "104"}]}, "Constraints": {}, "sku_mappings": [{"sku": "PL002", "combination": ["101", "102", "103", "104"]}]}</t>
+    <t>{
+"Power": "7W",
+"Color Temperature": "6000K",
+"Voltage": "12V",
+"IP Rating": "IP68",
+"SKU": "PL002"
+}</t>
   </si>
   <si>
     <t>pool light, 6000k, ip68 waterproof, 7w led, 12v lighting, aquatic light</t>
@@ -393,7 +368,7 @@
     <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -870,24 +845,24 @@
 1. Global Core Fields (Every "&amp;"SKU must have these):
 - Power (Example 1.2W, 7W)
 - Light Color (Example Warm White)
-- CCT (Example 3000K)
+- Color Temperature (Example 3000K)
 - Voltage (Example 20V, 12V/24V)
 - Current Type (Example AC/DC)
 - IP Rating (Example IP67, IP68)
 - Impact Strength (Example IK10)
-- Optics (Example S"&amp;"YS30°)
-- Finish (Example Black finish)
+- Opt"&amp;"ics (Example SYS30°)
+- Finish (Example Black)
 ### STRICT OUTPUT RULES
 1. Output ONLY the corresponding labels mentioned above separated by pipes ('|'). 
 2. Do not include the values in your output.
-3. Do not include any conversational text, introductory remarks"&amp;", or markdown formatting blocks.
+3. Do not include any conversational text, introductory "&amp;"remarks, or markdown formatting blocks.
 4. The number of labels in your output must exactly match the number of values provided in the input.
 ---
 ### FEW-SHOT EXAMPLES
 #### Example 1 (Standard Neon Strip)
-Input: 1.2W | SYM30° | 3000K | IP67 | IK10
-Output: Pow"&amp;"er|Optics|CCT|IP Rating|Impact Strength
-Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black finish
+Input: 1.2W | SYM 30° | 3000K | IP67 | IK10
+Out"&amp;"put: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black
 Output: Power | Light Color | Current Type | IP Rating | Finish
 ---
 ### YOUR TASK
@@ -898,7 +873,27 @@
         <v>37</v>
       </c>
       <c r="P2" s="13" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Using the labels""&amp;N2&amp;"" and values ""&amp;M2&amp;"" separated by character '|' and Using ""&amp;L2&amp;"" and key as 'SKU', Create a JSON object"")"),"{""Power"": ""7W"", ""Light Color"": ""Warm White"", ""Voltage"": ""12V/24V"", ""Current Type"": ""AC/DC"", ""IP Rating"": ""IP67"", ""Finish"": ""Black"", ""SKU"": ""GL001""}")</f>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a data processing assistant that converts delimited text into structured JSON.
+Task: Convert the provided pipe-delimited (|) header and value lines into a valid JSON object or array of objects.
+Instructions:
+- Clean both keys and values by "&amp;"trimming leading and trailing whitespace.
+- Remove any index prefix from the value string (e.g., convert 1.2W from 1.2W  or 1.2W without leading list numbers).
+- Map each key from Line 1 to its corresponding value in Line 2.
+- Output only valid, properly "&amp;"formatted JSON with no surrounding commentary or explanation.
+Example:
+Keys: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Values: 1.2W | SYM 30° | 4000K | IP67 | IK10
+SKU Code: HRS001
+Example Output:
+{
+  """"Power"""": """"1.2W"""",
+  """"Op"&amp;"tics"""": """"SYM 30°"""",
+  """"Color Temperature"""": """"4000K"""",
+  """"IP Rating"""": """"IP67"""",
+  """"Impact Strength"""": """"IK10"""",
+  """"SKU"""": """"HRS001""""
+}
+Generate JSON for the Keys: ""&amp;O2&amp;"", Values: ""&amp;M2&amp; "" and SKU Code: ""&amp;L2"&amp;")"),"{""Power"": ""7W"", ""Light Color"": ""Warm White"", ""Voltage"": ""12V/24V"", ""Current Type"": ""AC/DC"", ""IP Rating"": ""IP67"", ""Finish"": ""Black"", ""SKU"": ""GL001""}")</f>
         <v>{"Power": "7W", "Light Color": "Warm White", "Voltage": "12V/24V", "Current Type": "AC/DC", "IP Rating": "IP67", "Finish": "Black", "SKU": "GL001"}</v>
       </c>
       <c r="Q2" s="14" t="s">
@@ -921,45 +916,45 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a product catalog configuration expert. Your task is to analyze a list of valid product variant combinations (provided as JSON lines/objects) and generate two JSON structures: """"Options"""" and """"Constraints"""".
 ### Instructions:
 1. **"&amp;"Extract Options:**
-   - Group all unique values by their attribute keys (e.g., Power, Optics, CCT, IP Rating, Impact Strength).
-   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and incrementing by 1 in "&amp;"the order they appear.
+   - Group all unique values by their attribute keys (e.g., Power, Optics, Color Temperature, IP Rating, Impact Strength).
+   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and increme"&amp;"nting by 1 in the order they appear.
    - Format each attribute as an array of objects: `[{""""name"""": """"VALUE"""", """"id"""": """"ID""""}]`.
 2. **Determine Constraints (Incompatibilities):**
-   - Identify attribute pairs that are impossible or missing from the v"&amp;"alid combinations.
+   - Identify attribute pairs that are impossible or miss"&amp;"ing from the valid combinations.
    - Specifically, map an ID of an Option Value to an array of Option Value IDs that **cannot** be selected with it.
    - Output constraints in the format: `""""OPTION_ID"""": [INCOMPATIBLE_OPTION_ID]`.
-   - Only list meaningful non-emp"&amp;"ty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
+   - Only list mean"&amp;"ingful non-empty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
 3. **Determine sku_mappings:**
-   - Identify the valid combination and create a array with sku and combination containing array of options ID
-4. **O"&amp;"utput Format:**
+   - Identify the valid combination and create a array with sku and combination containing array of optio"&amp;"ns ID
+4. **Output Format:**
    - Return strictly valid JSON containing two root keys: """"Options"""", """"Constraints"""" and """"sku_mappings"""".
    - Do not wrap the JSON in conversational filler text.
 ---
 ### Example Input:
-{""""SKU"""":""""HRS001"""", """"Pow"&amp;"er"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""""&amp;": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Stre"&amp;"ngth"""": """"IK10""""}
-{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS005"""", """"Power"""&amp;""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS00"&amp;"1"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""":"&amp;" """"SYM30°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"300"&amp;"0K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact"&amp;" Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS005"""", """"Power"""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
 ### Example Output:
-{
+"&amp;"{
   """"Options"""": {
     """"Power"""": [
-      {""""name"""": """"1.2W"""", """""&amp;"id"""": """"101""""}
+      {""""name"""": """"1.2W"""", """"id"""": """"101""""}
     ],
     """"Optics"""": [
       {""""name"""": """"SYM30°"""", """"id"""": """"102""""},
-      {""""name"""": """"SYM60°"""", """"id"""": """"103""""},
+      {""""name"""": """"SYM60°"""", """"id"""": """"103"""&amp;"""},
       {""""name"""": """"ASYM50°"""", """"id"""": """"104""""}
     ],
-    """"C"&amp;"CT"""": [
+    """"Color Temperature"""": [
       {""""name"""": """"3000K"""", """"id"""": """"105""""},
       {""""name"""": """"4000K"""", """"id"""": """"106""""}
     ],
-    """"IP Rating"""": [
+    """"IP Rating"&amp;""""": [
       {""""name"""": """"IP67"""", """"id"""": """"107""""}
     ],
-    """"Impact Strength"&amp;""""": [
+    """"Impact Strength"""": [
       {""""name"""": """"IK10"""", """"id"""": """"108""""}
     ]
   },
@@ -967,72 +962,16 @@
     """"104"""": [106]
   },
 """"sku_mappings"""": [
-      { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+ "&amp;"     { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS002"""", """"combination"""": [""""101"""", """"102"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+  "&amp;"    { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS004"""", """"combination"""": [""""101"""", """"103"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+   "&amp;"   { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS006"""", """"combination"""": [""""101"""", """"104"""", """"106"""", """"107"""", """"108""""] }
-    ]
+    ]"&amp;"
 }
-Process the following product variant combinations and output the """"Options"""" and """"C"&amp;"onstraints"""" JSON:"", Q2)"),"{
-""Options"": {
-""Power"": [
-{""name"": ""7W"", ""id"": ""101""}
-],
-""Light Color"": [
-{""name"": ""Warm White"", ""id"": ""102""}
-],
-""Voltage"": [
-{""name"": ""12V/24V"", ""id"": ""103""}
-],
-""Current Type"": [
-{""name"": ""AC/DC"", ""id"": ""104""}
-],"&amp;"
-""IP Rating"": [
-{""name"": ""IP67"", ""id"": ""105""}
-],
-""Finish"": [
-{""name"": ""Black"", ""id"": ""106""}
-]
-},
-""Constraints"": {},
-""sku_mappings"": [
-{
-""sku"": ""GL001"",
-""combination"": [""101"", ""102"", ""103"", ""104"", ""105"", ""106""]
-}
-]"&amp;"
-}")</f>
-        <v>{
-"Options": {
-"Power": [
-{"name": "7W", "id": "101"}
-],
-"Light Color": [
-{"name": "Warm White", "id": "102"}
-],
-"Voltage": [
-{"name": "12V/24V", "id": "103"}
-],
-"Current Type": [
-{"name": "AC/DC", "id": "104"}
-],
-"IP Rating": [
-{"name": "IP67", "id": "105"}
-],
-"Finish": [
-{"name": "Black", "id": "106"}
-]
-},
-"Constraints": {},
-"sku_mappings": [
-{
-"sku": "GL001",
-"combination": ["101", "102", "103", "104", "105", "106"]
-}
-]
-}</v>
+Process the following product variant combinations and output the """"Options"""", """"Constraints"""" and """"sku_mappings"""" JSON:"", Q2)"),"{""Options"": {""Power"": [{""name"": ""7W"", ""id"": ""101""}], ""Light Color"": [{""name"": ""Warm White"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V/24V"", ""id"": ""103""}], ""Current Type"": [{""name"": ""AC/DC"", ""id"": ""104""}], ""IP Rati"&amp;"ng"": [{""name"": ""IP67"", ""id"": ""105""}], ""Finish"": [{""name"": ""Black"", ""id"": ""106""}]}, ""Constraints"": {}, ""sku_mappings"": [{""sku"": ""GL001"", ""combination"": [""101"", ""102"", ""103"", ""104"", ""105"", ""106""]}]}")</f>
+        <v>{"Options": {"Power": [{"name": "7W", "id": "101"}], "Light Color": [{"name": "Warm White", "id": "102"}], "Voltage": [{"name": "12V/24V", "id": "103"}], "Current Type": [{"name": "AC/DC", "id": "104"}], "IP Rating": [{"name": "IP67", "id": "105"}], "Finish": [{"name": "Black", "id": "106"}]}, "Constraints": {}, "sku_mappings": [{"sku": "GL001", "combination": ["101", "102", "103", "104", "105", "106"]}]}</v>
       </c>
       <c r="U2" s="16" t="s">
         <v>39</v>
@@ -1111,24 +1050,24 @@
 1. Global Core Fields (Every "&amp;"SKU must have these):
 - Power (Example 1.2W, 7W)
 - Light Color (Example Warm White)
-- CCT (Example 3000K)
+- Color Temperature (Example 3000K)
 - Voltage (Example 20V, 12V/24V)
 - Current Type (Example AC/DC)
 - IP Rating (Example IP67, IP68)
 - Impact Strength (Example IK10)
-- Optics (Example S"&amp;"YS30°)
-- Finish (Example Black finish)
+- Opt"&amp;"ics (Example SYS30°)
+- Finish (Example Black)
 ### STRICT OUTPUT RULES
 1. Output ONLY the corresponding labels mentioned above separated by pipes ('|'). 
 2. Do not include the values in your output.
-3. Do not include any conversational text, introductory remarks"&amp;", or markdown formatting blocks.
+3. Do not include any conversational text, introductory "&amp;"remarks, or markdown formatting blocks.
 4. The number of labels in your output must exactly match the number of values provided in the input.
 ---
 ### FEW-SHOT EXAMPLES
 #### Example 1 (Standard Neon Strip)
-Input: 1.2W | SYM30° | 3000K | IP67 | IK10
-Output: Pow"&amp;"er|Optics|CCT|IP Rating|Impact Strength
-Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black finish
+Input: 1.2W | SYM 30° | 3000K | IP67 | IK10
+Out"&amp;"put: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black
 Output: Power | Light Color | Current Type | IP Rating | Finish
 ---
 ### YOUR TASK
@@ -1139,7 +1078,27 @@
         <v>37</v>
       </c>
       <c r="P3" s="13" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Using the labels""&amp;N3&amp;"" and values ""&amp;M3&amp;"" separated by character '|' and Using ""&amp;L3&amp;"" and key as 'SKU', Create a JSON object"")"),"{""Power"": ""12W"", ""Light Color"": ""Warm White"", ""Voltage"": ""12V/24V"", ""Current Type"": ""AC/DC"", ""IP Rating"": ""IP67"", ""Finish"": ""Black"", ""SKU"": ""GL003""}")</f>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a data processing assistant that converts delimited text into structured JSON.
+Task: Convert the provided pipe-delimited (|) header and value lines into a valid JSON object or array of objects.
+Instructions:
+- Clean both keys and values by "&amp;"trimming leading and trailing whitespace.
+- Remove any index prefix from the value string (e.g., convert 1.2W from 1.2W  or 1.2W without leading list numbers).
+- Map each key from Line 1 to its corresponding value in Line 2.
+- Output only valid, properly "&amp;"formatted JSON with no surrounding commentary or explanation.
+Example:
+Keys: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Values: 1.2W | SYM 30° | 4000K | IP67 | IK10
+SKU Code: HRS001
+Example Output:
+{
+  """"Power"""": """"1.2W"""",
+  """"Op"&amp;"tics"""": """"SYM 30°"""",
+  """"Color Temperature"""": """"4000K"""",
+  """"IP Rating"""": """"IP67"""",
+  """"Impact Strength"""": """"IK10"""",
+  """"SKU"""": """"HRS001""""
+}
+Generate JSON for the Keys: ""&amp;O3&amp;"", Values: ""&amp;M3&amp; "" and SKU Code: ""&amp;L3"&amp;")"),"{""Power"": ""12W"", ""Light Color"": ""Warm White"", ""Voltage"": ""12V/24V"", ""Current Type"": ""AC/DC"", ""IP Rating"": ""IP67"", ""Finish"": ""Black"", ""SKU"": ""GL003""}")</f>
         <v>{"Power": "12W", "Light Color": "Warm White", "Voltage": "12V/24V", "Current Type": "AC/DC", "IP Rating": "IP67", "Finish": "Black", "SKU": "GL003"}</v>
       </c>
       <c r="Q3" s="14" t="s">
@@ -1162,45 +1121,45 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a product catalog configuration expert. Your task is to analyze a list of valid product variant combinations (provided as JSON lines/objects) and generate two JSON structures: """"Options"""" and """"Constraints"""".
 ### Instructions:
 1. **"&amp;"Extract Options:**
-   - Group all unique values by their attribute keys (e.g., Power, Optics, CCT, IP Rating, Impact Strength).
-   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and incrementing by 1 in "&amp;"the order they appear.
+   - Group all unique values by their attribute keys (e.g., Power, Optics, Color Temperature, IP Rating, Impact Strength).
+   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and increme"&amp;"nting by 1 in the order they appear.
    - Format each attribute as an array of objects: `[{""""name"""": """"VALUE"""", """"id"""": """"ID""""}]`.
 2. **Determine Constraints (Incompatibilities):**
-   - Identify attribute pairs that are impossible or missing from the v"&amp;"alid combinations.
+   - Identify attribute pairs that are impossible or miss"&amp;"ing from the valid combinations.
    - Specifically, map an ID of an Option Value to an array of Option Value IDs that **cannot** be selected with it.
    - Output constraints in the format: `""""OPTION_ID"""": [INCOMPATIBLE_OPTION_ID]`.
-   - Only list meaningful non-emp"&amp;"ty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
+   - Only list mean"&amp;"ingful non-empty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
 3. **Determine sku_mappings:**
-   - Identify the valid combination and create a array with sku and combination containing array of options ID
-4. **O"&amp;"utput Format:**
+   - Identify the valid combination and create a array with sku and combination containing array of optio"&amp;"ns ID
+4. **Output Format:**
    - Return strictly valid JSON containing two root keys: """"Options"""", """"Constraints"""" and """"sku_mappings"""".
    - Do not wrap the JSON in conversational filler text.
 ---
 ### Example Input:
-{""""SKU"""":""""HRS001"""", """"Pow"&amp;"er"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""""&amp;": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Stre"&amp;"ngth"""": """"IK10""""}
-{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS005"""", """"Power"""&amp;""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS00"&amp;"1"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""":"&amp;" """"SYM30°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"300"&amp;"0K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact"&amp;" Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS005"""", """"Power"""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
 ### Example Output:
-{
+"&amp;"{
   """"Options"""": {
     """"Power"""": [
-      {""""name"""": """"1.2W"""", """""&amp;"id"""": """"101""""}
+      {""""name"""": """"1.2W"""", """"id"""": """"101""""}
     ],
     """"Optics"""": [
       {""""name"""": """"SYM30°"""", """"id"""": """"102""""},
-      {""""name"""": """"SYM60°"""", """"id"""": """"103""""},
+      {""""name"""": """"SYM60°"""", """"id"""": """"103"""&amp;"""},
       {""""name"""": """"ASYM50°"""", """"id"""": """"104""""}
     ],
-    """"C"&amp;"CT"""": [
+    """"Color Temperature"""": [
       {""""name"""": """"3000K"""", """"id"""": """"105""""},
       {""""name"""": """"4000K"""", """"id"""": """"106""""}
     ],
-    """"IP Rating"""": [
+    """"IP Rating"&amp;""""": [
       {""""name"""": """"IP67"""", """"id"""": """"107""""}
     ],
-    """"Impact Strength"&amp;""""": [
+    """"Impact Strength"""": [
       {""""name"""": """"IK10"""", """"id"""": """"108""""}
     ]
   },
@@ -1208,15 +1167,15 @@
     """"104"""": [106]
   },
 """"sku_mappings"""": [
-      { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+ "&amp;"     { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS002"""", """"combination"""": [""""101"""", """"102"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+  "&amp;"    { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS004"""", """"combination"""": [""""101"""", """"103"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+   "&amp;"   { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS006"""", """"combination"""": [""""101"""", """"104"""", """"106"""", """"107"""", """"108""""] }
-    ]
+    ]"&amp;"
 }
-Process the following product variant combinations and output the """"Options"""" and """"C"&amp;"onstraints"""" JSON:"", Q3)"),"{""Options"": {""Power"": [{""name"": ""12W"", ""id"": ""101""}], ""Light Color"": [{""name"": ""Warm White"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V/24V"", ""id"": ""103""}], ""Current Type"": [{""name"": ""AC/DC"", ""id"": ""104""}], ""IP Rat"&amp;"ing"": [{""name"": ""IP67"", ""id"": ""105""}], ""Finish"": [{""name"": ""Black"", ""id"": ""106""}]}, ""Constraints"": {}, ""sku_mappings"": [{""sku"": ""GL003"", ""combination"": [""101"", ""102"", ""103"", ""104"", ""105"", ""106""]}]}")</f>
+Process the following product variant combinations and output the """"Options"""", """"Constraints"""" and """"sku_mappings"""" JSON:"", Q3)"),"{""Options"": {""Power"": [{""name"": ""12W"", ""id"": ""101""}], ""Light Color"": [{""name"": ""Warm White"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V/24V"", ""id"": ""103""}], ""Current Type"": [{""name"": ""AC/DC"", ""id"": ""104""}], ""IP Rat"&amp;"ing"": [{""name"": ""IP67"", ""id"": ""105""}], ""Finish"": [{""name"": ""Black"", ""id"": ""106""}]}, ""Constraints"": {}, ""sku_mappings"": [{""sku"": ""GL003"", ""combination"": [""101"", ""102"", ""103"", ""104"", ""105"", ""106""]}]}")</f>
         <v>{"Options": {"Power": [{"name": "12W", "id": "101"}], "Light Color": [{"name": "Warm White", "id": "102"}], "Voltage": [{"name": "12V/24V", "id": "103"}], "Current Type": [{"name": "AC/DC", "id": "104"}], "IP Rating": [{"name": "IP67", "id": "105"}], "Finish": [{"name": "Black", "id": "106"}]}, "Constraints": {}, "sku_mappings": [{"sku": "GL003", "combination": ["101", "102", "103", "104", "105", "106"]}]}</v>
       </c>
       <c r="U3" s="16" t="s">
@@ -1296,24 +1255,24 @@
 1. Global Core Fields (Every "&amp;"SKU must have these):
 - Power (Example 1.2W, 7W)
 - Light Color (Example Warm White)
-- CCT (Example 3000K)
+- Color Temperature (Example 3000K)
 - Voltage (Example 20V, 12V/24V)
 - Current Type (Example AC/DC)
 - IP Rating (Example IP67, IP68)
 - Impact Strength (Example IK10)
-- Optics (Example S"&amp;"YS30°)
-- Finish (Example Black finish)
+- Opt"&amp;"ics (Example SYS30°)
+- Finish (Example Black)
 ### STRICT OUTPUT RULES
 1. Output ONLY the corresponding labels mentioned above separated by pipes ('|'). 
 2. Do not include the values in your output.
-3. Do not include any conversational text, introductory remarks"&amp;", or markdown formatting blocks.
+3. Do not include any conversational text, introductory "&amp;"remarks, or markdown formatting blocks.
 4. The number of labels in your output must exactly match the number of values provided in the input.
 ---
 ### FEW-SHOT EXAMPLES
 #### Example 1 (Standard Neon Strip)
-Input: 1.2W | SYM30° | 3000K | IP67 | IK10
-Output: Pow"&amp;"er|Optics|CCT|IP Rating|Impact Strength
-Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black finish
+Input: 1.2W | SYM 30° | 3000K | IP67 | IK10
+Out"&amp;"put: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black
 Output: Power | Light Color | Current Type | IP Rating | Finish
 ---
 ### YOUR TASK
@@ -1324,7 +1283,27 @@
         <v>37</v>
       </c>
       <c r="P4" s="13" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Using the labels""&amp;N4&amp;"" and values ""&amp;M4&amp;"" separated by character '|' and Using ""&amp;L4&amp;"" and key as 'SKU', Create a JSON object"")"),"{""Power"": ""3W"", ""Light Color"": ""Warm White"", ""Voltage"": ""12V/24V"", ""Current Type"": ""AC/DC"", ""IP Rating"": ""IP67"", ""Finish"": ""Black"", ""SKU"": ""GL005""}")</f>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a data processing assistant that converts delimited text into structured JSON.
+Task: Convert the provided pipe-delimited (|) header and value lines into a valid JSON object or array of objects.
+Instructions:
+- Clean both keys and values by "&amp;"trimming leading and trailing whitespace.
+- Remove any index prefix from the value string (e.g., convert 1.2W from 1.2W  or 1.2W without leading list numbers).
+- Map each key from Line 1 to its corresponding value in Line 2.
+- Output only valid, properly "&amp;"formatted JSON with no surrounding commentary or explanation.
+Example:
+Keys: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Values: 1.2W | SYM 30° | 4000K | IP67 | IK10
+SKU Code: HRS001
+Example Output:
+{
+  """"Power"""": """"1.2W"""",
+  """"Op"&amp;"tics"""": """"SYM 30°"""",
+  """"Color Temperature"""": """"4000K"""",
+  """"IP Rating"""": """"IP67"""",
+  """"Impact Strength"""": """"IK10"""",
+  """"SKU"""": """"HRS001""""
+}
+Generate JSON for the Keys: ""&amp;O4&amp;"", Values: ""&amp;M4&amp; "" and SKU Code: ""&amp;L4"&amp;")"),"{""Power"": ""3W"", ""Light Color"": ""Warm White"", ""Voltage"": ""12V/24V"", ""Current Type"": ""AC/DC"", ""IP Rating"": ""IP67"", ""Finish"": ""Black"", ""SKU"": ""GL005""}")</f>
         <v>{"Power": "3W", "Light Color": "Warm White", "Voltage": "12V/24V", "Current Type": "AC/DC", "IP Rating": "IP67", "Finish": "Black", "SKU": "GL005"}</v>
       </c>
       <c r="Q4" s="14" t="s">
@@ -1347,45 +1326,45 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a product catalog configuration expert. Your task is to analyze a list of valid product variant combinations (provided as JSON lines/objects) and generate two JSON structures: """"Options"""" and """"Constraints"""".
 ### Instructions:
 1. **"&amp;"Extract Options:**
-   - Group all unique values by their attribute keys (e.g., Power, Optics, CCT, IP Rating, Impact Strength).
-   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and incrementing by 1 in "&amp;"the order they appear.
+   - Group all unique values by their attribute keys (e.g., Power, Optics, Color Temperature, IP Rating, Impact Strength).
+   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and increme"&amp;"nting by 1 in the order they appear.
    - Format each attribute as an array of objects: `[{""""name"""": """"VALUE"""", """"id"""": """"ID""""}]`.
 2. **Determine Constraints (Incompatibilities):**
-   - Identify attribute pairs that are impossible or missing from the v"&amp;"alid combinations.
+   - Identify attribute pairs that are impossible or miss"&amp;"ing from the valid combinations.
    - Specifically, map an ID of an Option Value to an array of Option Value IDs that **cannot** be selected with it.
    - Output constraints in the format: `""""OPTION_ID"""": [INCOMPATIBLE_OPTION_ID]`.
-   - Only list meaningful non-emp"&amp;"ty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
+   - Only list mean"&amp;"ingful non-empty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
 3. **Determine sku_mappings:**
-   - Identify the valid combination and create a array with sku and combination containing array of options ID
-4. **O"&amp;"utput Format:**
+   - Identify the valid combination and create a array with sku and combination containing array of optio"&amp;"ns ID
+4. **Output Format:**
    - Return strictly valid JSON containing two root keys: """"Options"""", """"Constraints"""" and """"sku_mappings"""".
    - Do not wrap the JSON in conversational filler text.
 ---
 ### Example Input:
-{""""SKU"""":""""HRS001"""", """"Pow"&amp;"er"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""""&amp;": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Stre"&amp;"ngth"""": """"IK10""""}
-{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS005"""", """"Power"""&amp;""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS00"&amp;"1"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""":"&amp;" """"SYM30°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"300"&amp;"0K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact"&amp;" Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS005"""", """"Power"""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
 ### Example Output:
-{
+"&amp;"{
   """"Options"""": {
     """"Power"""": [
-      {""""name"""": """"1.2W"""", """""&amp;"id"""": """"101""""}
+      {""""name"""": """"1.2W"""", """"id"""": """"101""""}
     ],
     """"Optics"""": [
       {""""name"""": """"SYM30°"""", """"id"""": """"102""""},
-      {""""name"""": """"SYM60°"""", """"id"""": """"103""""},
+      {""""name"""": """"SYM60°"""", """"id"""": """"103"""&amp;"""},
       {""""name"""": """"ASYM50°"""", """"id"""": """"104""""}
     ],
-    """"C"&amp;"CT"""": [
+    """"Color Temperature"""": [
       {""""name"""": """"3000K"""", """"id"""": """"105""""},
       {""""name"""": """"4000K"""", """"id"""": """"106""""}
     ],
-    """"IP Rating"""": [
+    """"IP Rating"&amp;""""": [
       {""""name"""": """"IP67"""", """"id"""": """"107""""}
     ],
-    """"Impact Strength"&amp;""""": [
+    """"Impact Strength"""": [
       {""""name"""": """"IK10"""", """"id"""": """"108""""}
     ]
   },
@@ -1393,15 +1372,15 @@
     """"104"""": [106]
   },
 """"sku_mappings"""": [
-      { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+ "&amp;"     { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS002"""", """"combination"""": [""""101"""", """"102"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+  "&amp;"    { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS004"""", """"combination"""": [""""101"""", """"103"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+   "&amp;"   { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS006"""", """"combination"""": [""""101"""", """"104"""", """"106"""", """"107"""", """"108""""] }
-    ]
+    ]"&amp;"
 }
-Process the following product variant combinations and output the """"Options"""" and """"C"&amp;"onstraints"""" JSON:"", Q4)"),"{""Options"": {""Power"": [{""name"": ""3W"", ""id"": ""101""}], ""Light Color"": [{""name"": ""Warm White"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V/24V"", ""id"": ""103""}], ""Current Type"": [{""name"": ""AC/DC"", ""id"": ""104""}], ""IP Rati"&amp;"ng"": [{""name"": ""IP67"", ""id"": ""105""}], ""Finish"": [{""name"": ""Black"", ""id"": ""106""}]}, ""Constraints"": {}, ""sku_mappings"": [{""sku"": ""GL005"", ""combination"": [""101"", ""102"", ""103"", ""104"", ""105"", ""106""]}]}")</f>
+Process the following product variant combinations and output the """"Options"""", """"Constraints"""" and """"sku_mappings"""" JSON:"", Q4)"),"{""Options"": {""Power"": [{""name"": ""3W"", ""id"": ""101""}], ""Light Color"": [{""name"": ""Warm White"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V/24V"", ""id"": ""103""}], ""Current Type"": [{""name"": ""AC/DC"", ""id"": ""104""}], ""IP Rati"&amp;"ng"": [{""name"": ""IP67"", ""id"": ""105""}], ""Finish"": [{""name"": ""Black"", ""id"": ""106""}]}, ""Constraints"": {}, ""sku_mappings"": [{""sku"": ""GL005"", ""combination"": [""101"", ""102"", ""103"", ""104"", ""105"", ""106""]}]}")</f>
         <v>{"Options": {"Power": [{"name": "3W", "id": "101"}], "Light Color": [{"name": "Warm White", "id": "102"}], "Voltage": [{"name": "12V/24V", "id": "103"}], "Current Type": [{"name": "AC/DC", "id": "104"}], "IP Rating": [{"name": "IP67", "id": "105"}], "Finish": [{"name": "Black", "id": "106"}]}, "Constraints": {}, "sku_mappings": [{"sku": "GL005", "combination": ["101", "102", "103", "104", "105", "106"]}]}</v>
       </c>
       <c r="U4" s="16" t="s">
@@ -1481,36 +1460,56 @@
 1. Global Core Fields (Every "&amp;"SKU must have these):
 - Power (Example 1.2W, 7W)
 - Light Color (Example Warm White)
-- CCT (Example 3000K)
+- Color Temperature (Example 3000K)
 - Voltage (Example 20V, 12V/24V)
 - Current Type (Example AC/DC)
 - IP Rating (Example IP67, IP68)
 - Impact Strength (Example IK10)
-- Optics (Example S"&amp;"YS30°)
-- Finish (Example Black finish)
+- Opt"&amp;"ics (Example SYS30°)
+- Finish (Example Black)
 ### STRICT OUTPUT RULES
 1. Output ONLY the corresponding labels mentioned above separated by pipes ('|'). 
 2. Do not include the values in your output.
-3. Do not include any conversational text, introductory remarks"&amp;", or markdown formatting blocks.
+3. Do not include any conversational text, introductory "&amp;"remarks, or markdown formatting blocks.
 4. The number of labels in your output must exactly match the number of values provided in the input.
 ---
 ### FEW-SHOT EXAMPLES
 #### Example 1 (Standard Neon Strip)
-Input: 1.2W | SYM30° | 3000K | IP67 | IK10
-Output: Pow"&amp;"er|Optics|CCT|IP Rating|Impact Strength
-Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black finish
+Input: 1.2W | SYM 30° | 3000K | IP67 | IK10
+Out"&amp;"put: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black
 Output: Power | Light Color | Current Type | IP Rating | Finish
 ---
 ### YOUR TASK
-Generate output for the values text ""&amp;M5)"),"Power|CCT|Voltage|IP Rating")</f>
-        <v>Power|CCT|Voltage|IP Rating</v>
+Generate output for the values text ""&amp;M5)"),"Power|Color Temperature|Voltage|IP Rating")</f>
+        <v>Power|Color Temperature|Voltage|IP Rating</v>
       </c>
       <c r="O5" s="14" t="s">
         <v>61</v>
       </c>
       <c r="P5" s="13" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Using the labels""&amp;N5&amp;"" and values ""&amp;M5&amp;"" separated by character '|' and Using ""&amp;L5&amp;"" and key as 'SKU', Create a JSON object"")"),"{""Power"": ""7W"", ""CCT"": ""3000K"", ""Voltage"": ""12V"", ""IP Rating"": ""IP68"", ""SKU"": ""PL001""}")</f>
-        <v>{"Power": "7W", "CCT": "3000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL001"}</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a data processing assistant that converts delimited text into structured JSON.
+Task: Convert the provided pipe-delimited (|) header and value lines into a valid JSON object or array of objects.
+Instructions:
+- Clean both keys and values by "&amp;"trimming leading and trailing whitespace.
+- Remove any index prefix from the value string (e.g., convert 1.2W from 1.2W  or 1.2W without leading list numbers).
+- Map each key from Line 1 to its corresponding value in Line 2.
+- Output only valid, properly "&amp;"formatted JSON with no surrounding commentary or explanation.
+Example:
+Keys: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Values: 1.2W | SYM 30° | 4000K | IP67 | IK10
+SKU Code: HRS001
+Example Output:
+{
+  """"Power"""": """"1.2W"""",
+  """"Op"&amp;"tics"""": """"SYM 30°"""",
+  """"Color Temperature"""": """"4000K"""",
+  """"IP Rating"""": """"IP67"""",
+  """"Impact Strength"""": """"IK10"""",
+  """"SKU"""": """"HRS001""""
+}
+Generate JSON for the Keys: ""&amp;O5&amp;"", Values: ""&amp;M5&amp; "" and SKU Code: ""&amp;L5"&amp;")"),"{""Power"": ""7W"", ""Color Temperature"": ""3000K"", ""Voltage"": ""12V"", ""IP Rating"": ""IP68"", ""SKU"": ""PL001""}")</f>
+        <v>{"Power": "7W", "Color Temperature": "3000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL001"}</v>
       </c>
       <c r="Q5" s="14" t="s">
         <v>62</v>
@@ -1522,55 +1521,55 @@
 2. If a key has the same value across all objects, render it as a single primitive value (string/number).  
 3. If a key has multiple distinct values across the objects, combine them into an array containing only the unique values (deduplicated).  
 4. Ma"&amp;"intain a clean, properly formatted, and valid JSON structure.  
-Here is the input data:"", Q5)"),"{""Power"": ""7W"", ""CCT"": ""3000K"", ""Voltage"": ""12V"", ""IP Rating"": ""IP68"", ""SKU"": ""PL001""}")</f>
-        <v>{"Power": "7W", "CCT": "3000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL001"}</v>
+Here is the input data:"", Q5:Q6)"),"{""Power"": ""7W"", ""Color Temperature"": [""3000K"", ""6000K""], ""Voltage"": ""12V"", ""IP Rating"": ""IP68"", ""SKU"": [""PL001"", ""PL002""]}")</f>
+        <v>{"Power": "7W", "Color Temperature": ["3000K", "6000K"], "Voltage": "12V", "IP Rating": "IP68", "SKU": ["PL001", "PL002"]}</v>
       </c>
       <c r="S5" s="15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="T5" s="11" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a product catalog configuration expert. Your task is to analyze a list of valid product variant combinations (provided as JSON lines/objects) and generate two JSON structures: """"Options"""" and """"Constraints"""".
 ### Instructions:
 1. **"&amp;"Extract Options:**
-   - Group all unique values by their attribute keys (e.g., Power, Optics, CCT, IP Rating, Impact Strength).
-   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and incrementing by 1 in "&amp;"the order they appear.
+   - Group all unique values by their attribute keys (e.g., Power, Optics, Color Temperature, IP Rating, Impact Strength).
+   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and increme"&amp;"nting by 1 in the order they appear.
    - Format each attribute as an array of objects: `[{""""name"""": """"VALUE"""", """"id"""": """"ID""""}]`.
 2. **Determine Constraints (Incompatibilities):**
-   - Identify attribute pairs that are impossible or missing from the v"&amp;"alid combinations.
+   - Identify attribute pairs that are impossible or miss"&amp;"ing from the valid combinations.
    - Specifically, map an ID of an Option Value to an array of Option Value IDs that **cannot** be selected with it.
    - Output constraints in the format: `""""OPTION_ID"""": [INCOMPATIBLE_OPTION_ID]`.
-   - Only list meaningful non-emp"&amp;"ty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
+   - Only list mean"&amp;"ingful non-empty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
 3. **Determine sku_mappings:**
-   - Identify the valid combination and create a array with sku and combination containing array of options ID
-4. **O"&amp;"utput Format:**
+   - Identify the valid combination and create a array with sku and combination containing array of optio"&amp;"ns ID
+4. **Output Format:**
    - Return strictly valid JSON containing two root keys: """"Options"""", """"Constraints"""" and """"sku_mappings"""".
    - Do not wrap the JSON in conversational filler text.
 ---
 ### Example Input:
-{""""SKU"""":""""HRS001"""", """"Pow"&amp;"er"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""""&amp;": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Stre"&amp;"ngth"""": """"IK10""""}
-{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS005"""", """"Power"""&amp;""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS00"&amp;"1"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""":"&amp;" """"SYM30°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"300"&amp;"0K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"Color Temperature"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact"&amp;" Strength"""": """"IK10""""}
+{""""SKU"""":""""HRS005"""", """"Power"""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"Color Temperature"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
 ### Example Output:
-{
+"&amp;"{
   """"Options"""": {
     """"Power"""": [
-      {""""name"""": """"1.2W"""", """""&amp;"id"""": """"101""""}
+      {""""name"""": """"1.2W"""", """"id"""": """"101""""}
     ],
     """"Optics"""": [
       {""""name"""": """"SYM30°"""", """"id"""": """"102""""},
-      {""""name"""": """"SYM60°"""", """"id"""": """"103""""},
+      {""""name"""": """"SYM60°"""", """"id"""": """"103"""&amp;"""},
       {""""name"""": """"ASYM50°"""", """"id"""": """"104""""}
     ],
-    """"C"&amp;"CT"""": [
+    """"Color Temperature"""": [
       {""""name"""": """"3000K"""", """"id"""": """"105""""},
       {""""name"""": """"4000K"""", """"id"""": """"106""""}
     ],
-    """"IP Rating"""": [
+    """"IP Rating"&amp;""""": [
       {""""name"""": """"IP67"""", """"id"""": """"107""""}
     ],
-    """"Impact Strength"&amp;""""": [
+    """"Impact Strength"""": [
       {""""name"""": """"IK10"""", """"id"""": """"108""""}
     ]
   },
@@ -1578,40 +1577,40 @@
     """"104"""": [106]
   },
 """"sku_mappings"""": [
-      { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+ "&amp;"     { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS002"""", """"combination"""": [""""101"""", """"102"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+  "&amp;"    { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS004"""", """"combination"""": [""""101"""", """"103"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", "&amp;"""""107"""", """"108""""] },
+   "&amp;"   { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", """"107"""", """"108""""] },
       { """"sku"""": """"HRS006"""", """"combination"""": [""""101"""", """"104"""", """"106"""", """"107"""", """"108""""] }
-    ]
+    ]"&amp;"
 }
-Process the following product variant combinations and output the """"Options"""" and """"C"&amp;"onstraints"""" JSON:"", Q5)"),"{""Options"": {""Power"": [{""name"": ""7W"", ""id"": ""101""}], ""CCT"": [{""name"": ""3000K"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V"", ""id"": ""103""}], ""IP Rating"": [{""name"": ""IP68"", ""id"": ""104""}]}, ""Constraints"": {}, ""sku_ma"&amp;"ppings"": [{""sku"": ""PL001"", ""combination"": [""101"", ""102"", ""103"", ""104""]}]}")</f>
-        <v>{"Options": {"Power": [{"name": "7W", "id": "101"}], "CCT": [{"name": "3000K", "id": "102"}], "Voltage": [{"name": "12V", "id": "103"}], "IP Rating": [{"name": "IP68", "id": "104"}]}, "Constraints": {}, "sku_mappings": [{"sku": "PL001", "combination": ["101", "102", "103", "104"]}]}</v>
+Process the following product variant combinations and output the """"Options"""", """"Constraints"""" and """"sku_mappings"""" JSON:"", Q5:Q6)"),"{""Options"": {""Power"": [{""name"": ""7W"", ""id"": ""101""}], ""Color Temperature"": [{""name"": ""3000K"", ""id"": ""102""}, {""name"": ""6000K"", ""id"": ""103""}], ""Voltage"": [{""name"": ""12V"", ""id"": ""104""}], ""IP Rating"": [{""name"": ""IP6"&amp;"8"", ""id"": ""105""}]}, ""Constraints"": {}, ""sku_mappings"": [{""sku"": ""PL001"", ""combination"": [""101"", ""102"", ""104"", ""105""]}, {""sku"": ""PL002"", ""combination"": [""101"", ""103"", ""104"", ""105""]}]}")</f>
+        <v>{"Options": {"Power": [{"name": "7W", "id": "101"}], "Color Temperature": [{"name": "3000K", "id": "102"}, {"name": "6000K", "id": "103"}], "Voltage": [{"name": "12V", "id": "104"}], "IP Rating": [{"name": "IP68", "id": "105"}]}, "Constraints": {}, "sku_mappings": [{"sku": "PL001", "combination": ["101", "102", "104", "105"]}, {"sku": "PL002", "combination": ["101", "103", "104", "105"]}]}</v>
       </c>
       <c r="U5" s="16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="V5" s="17" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract options object from the json"", U5)"),"{""Power"": [{""name"": ""7W"", ""id"": ""101""}], ""CCT"": [{""name"": ""3000K"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V"", ""id"": ""103""}], ""IP Rating"": [{""name"": ""IP68"", ""id"": ""104""}]}")</f>
-        <v>{"Power": [{"name": "7W", "id": "101"}], "CCT": [{"name": "3000K", "id": "102"}], "Voltage": [{"name": "12V", "id": "103"}], "IP Rating": [{"name": "IP68", "id": "104"}]}</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract options object from the json"", U5)"),"{""Power"": [{""name"": ""7W"", ""id"": ""101""}], ""Color Temperature"": [{""name"": ""3000K"", ""id"": ""102""}, {""name"": ""6000K"", ""id"": ""103""}], ""Voltage"": [{""name"": ""12V"", ""id"": ""104""}], ""IP Rating"": [{""name"": ""IP68"", ""id"": "&amp;"""105""}]}")</f>
+        <v>{"Power": [{"name": "7W", "id": "101"}], "Color Temperature": [{"name": "3000K", "id": "102"}, {"name": "6000K", "id": "103"}], "Voltage": [{"name": "12V", "id": "104"}], "IP Rating": [{"name": "IP68", "id": "105"}]}</v>
       </c>
       <c r="W5" s="17" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract constraints object from the json"", U5)"),"{}")</f>
         <v>{}</v>
       </c>
       <c r="X5" s="17" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract sku_mappings object from the json"", U5)"),"[{""sku"": ""PL001"", ""combination"": [""101"", ""102"", ""103"", ""104""]}]")</f>
-        <v>[{"sku": "PL001", "combination": ["101", "102", "103", "104"]}]</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract sku_mappings object from the json"", U5)"),"[{""sku"": ""PL001"", ""combination"": [""101"", ""102"", ""104"", ""105""]}, {""sku"": ""PL002"", ""combination"": [""101"", ""103"", ""104"", ""105""]}]")</f>
+        <v>[{"sku": "PL001", "combination": ["101", "102", "104", "105"]}, {"sku": "PL002", "combination": ["101", "103", "104", "105"]}]</v>
       </c>
       <c r="Y5" s="15" t="s">
         <v>40</v>
       </c>
       <c r="Z5" s="15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AA5" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AB5" s="18"/>
       <c r="AC5" s="19" t="str">
@@ -1619,43 +1618,23 @@
         <v>pool light, underwater lighting, IP68 waterproof, 3000K warm white, low voltage LED, aquatic illumination</v>
       </c>
       <c r="AD5" s="18" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" ht="37.5" customHeight="1">
-      <c r="A6" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Give me a paragraph marketing spiel for this product, no tech specs just marketing fluff "")"),"Dive into an enchanting oasis of light and luxury with our premium pool illumination solution. Designed to effortlessly elevate your outdoor experience, it bathes your aquatic retreat in a warm, sophisticated radiance that creates an unparalleled ambiance"&amp;". Perfect for those with a discerning eye for discreet elegance and refined architectural detail, this lighting masterpiece transforms ordinary evenings into a breathtaking visual journey, adding both captivating allure and a profound sense of serenity to"&amp;" your home.")</f>
-        <v>Dive into an enchanting oasis of light and luxury with our premium pool illumination solution. Designed to effortlessly elevate your outdoor experience, it bathes your aquatic retreat in a warm, sophisticated radiance that creates an unparalleled ambiance. Perfect for those with a discerning eye for discreet elegance and refined architectural detail, this lighting masterpiece transforms ordinary evenings into a breathtaking visual journey, adding both captivating allure and a profound sense of serenity to your home.</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Give me a paragraph marketing spiel for this product, no tech specs just marketing fluff under 180 characters "")"),"Transform your pool into a breathtaking oasis. Elevate your outdoor space with a sophisticated glow that brings enchanting elegance and serene luxury to every evening.")</f>
-        <v>Transform your pool into a breathtaking oasis. Elevate your outdoor space with a sophisticated glow that brings enchanting elegance and serene luxury to every evening.</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>68</v>
-      </c>
+    </row>
+    <row r="6" ht="37.5" customHeight="1">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="10"/>
       <c r="J6" s="10"/>
       <c r="K6" s="10"/>
       <c r="L6" s="12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M6" s="12" t="s">
         <v>69</v>
@@ -1666,137 +1645,87 @@
 1. Global Core Fields (Every "&amp;"SKU must have these):
 - Power (Example 1.2W, 7W)
 - Light Color (Example Warm White)
-- CCT (Example 3000K)
+- Color Temperature (Example 3000K)
 - Voltage (Example 20V, 12V/24V)
 - Current Type (Example AC/DC)
 - IP Rating (Example IP67, IP68)
 - Impact Strength (Example IK10)
-- Optics (Example S"&amp;"YS30°)
-- Finish (Example Black finish)
+- Opt"&amp;"ics (Example SYS30°)
+- Finish (Example Black)
 ### STRICT OUTPUT RULES
 1. Output ONLY the corresponding labels mentioned above separated by pipes ('|'). 
 2. Do not include the values in your output.
-3. Do not include any conversational text, introductory remarks"&amp;", or markdown formatting blocks.
+3. Do not include any conversational text, introductory "&amp;"remarks, or markdown formatting blocks.
 4. The number of labels in your output must exactly match the number of values provided in the input.
 ---
 ### FEW-SHOT EXAMPLES
 #### Example 1 (Standard Neon Strip)
-Input: 1.2W | SYM30° | 3000K | IP67 | IK10
-Output: Pow"&amp;"er|Optics|CCT|IP Rating|Impact Strength
-Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black finish
+Input: 1.2W | SYM 30° | 3000K | IP67 | IK10
+Out"&amp;"put: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Input: 7W | Warm White | 12V/24V | AC/DC | IP67 | Black
 Output: Power | Light Color | Current Type | IP Rating | Finish
 ---
 ### YOUR TASK
-Generate output for the values text ""&amp;M6)"),"Power|CCT|Voltage|IP Rating")</f>
-        <v>Power|CCT|Voltage|IP Rating</v>
+Generate output for the values text ""&amp;M6)"),"Power|Color Temperature|Voltage|IP Rating")</f>
+        <v>Power|Color Temperature|Voltage|IP Rating</v>
       </c>
       <c r="O6" s="14" t="s">
         <v>61</v>
       </c>
       <c r="P6" s="13" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Using the labels""&amp;N6&amp;"" and values ""&amp;M6&amp;"" separated by character '|' and Using ""&amp;L6&amp;"" and key as 'SKU', Create a JSON object"")"),"{""Power"": ""7W"", ""CCT"": ""6000K"", ""Voltage"": ""12V"", ""IP Rating"": ""IP68"", ""SKU"": ""PL002""}")</f>
-        <v>{"Power": "7W", "CCT": "6000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL002"}</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a data processing assistant that converts delimited text into structured JSON.
+Task: Convert the provided pipe-delimited (|) header and value lines into a valid JSON object or array of objects.
+Instructions:
+- Clean both keys and values by "&amp;"trimming leading and trailing whitespace.
+- Remove any index prefix from the value string (e.g., convert 1.2W from 1.2W  or 1.2W without leading list numbers).
+- Map each key from Line 1 to its corresponding value in Line 2.
+- Output only valid, properly "&amp;"formatted JSON with no surrounding commentary or explanation.
+Example:
+Keys: Power|Optics|Color Temperature|IP Rating|Impact Strength
+Values: 1.2W | SYM 30° | 4000K | IP67 | IK10
+SKU Code: HRS001
+Example Output:
+{
+  """"Power"""": """"1.2W"""",
+  """"Op"&amp;"tics"""": """"SYM 30°"""",
+  """"Color Temperature"""": """"4000K"""",
+  """"IP Rating"""": """"IP67"""",
+  """"Impact Strength"""": """"IK10"""",
+  """"SKU"""": """"HRS001""""
+}
+Generate JSON for the Keys: ""&amp;O6&amp;"", Values: ""&amp;M6&amp; "" and SKU Code: ""&amp;L6"&amp;")"),"{
+""Power"": ""7W"",
+""Color Temperature"": ""6000K"",
+""Voltage"": ""12V"",
+""IP Rating"": ""IP68"",
+""SKU"": ""PL002""
+}")</f>
+        <v>{
+"Power": "7W",
+"Color Temperature": "6000K",
+"Voltage": "12V",
+"IP Rating": "IP68",
+"SKU": "PL002"
+}</v>
       </c>
       <c r="Q6" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="R6" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Act as a JSON Data Processing Specialist. I have a series of individual JSON objects that need to be merged into a single consolidated JSON object.  
-Please merge them following these rules:  
-1. Preserve all unique keys present across the objects. "&amp;" 
-2. If a key has the same value across all objects, render it as a single primitive value (string/number).  
-3. If a key has multiple distinct values across the objects, combine them into an array containing only the unique values (deduplicated).  
-4. Ma"&amp;"intain a clean, properly formatted, and valid JSON structure.  
-Here is the input data:"", Q6)"),"{""Power"": ""7W"", ""CCT"": ""6000K"", ""Voltage"": ""12V"", ""IP Rating"": ""IP68"", ""SKU"": ""PL002""}")</f>
-        <v>{"Power": "7W", "CCT": "6000K", "Voltage": "12V", "IP Rating": "IP68", "SKU": "PL002"}</v>
-      </c>
-      <c r="S6" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="T6" s="11" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""You are a product catalog configuration expert. Your task is to analyze a list of valid product variant combinations (provided as JSON lines/objects) and generate two JSON structures: """"Options"""" and """"Constraints"""".
-### Instructions:
-1. **"&amp;"Extract Options:**
-   - Group all unique values by their attribute keys (e.g., Power, Optics, CCT, IP Rating, Impact Strength).
-   - Assign a unique sequential integer string ID to every attribute value, starting from """"101"""" and incrementing by 1 in "&amp;"the order they appear.
-   - Format each attribute as an array of objects: `[{""""name"""": """"VALUE"""", """"id"""": """"ID""""}]`.
-2. **Determine Constraints (Incompatibilities):**
-   - Identify attribute pairs that are impossible or missing from the v"&amp;"alid combinations.
-   - Specifically, map an ID of an Option Value to an array of Option Value IDs that **cannot** be selected with it.
-   - Output constraints in the format: `""""OPTION_ID"""": [INCOMPATIBLE_OPTION_ID]`.
-   - Only list meaningful non-emp"&amp;"ty constraints. Express constraints using the primary driving factor (e.g., optic limitation over CCT).
-3. **Determine sku_mappings:**
-   - Identify the valid combination and create a array with sku and combination containing array of options ID
-4. **O"&amp;"utput Format:**
-   - Return strictly valid JSON containing two root keys: """"Options"""", """"Constraints"""" and """"sku_mappings"""".
-   - Do not wrap the JSON in conversational filler text.
----
-### Example Input:
-{""""SKU"""":""""HRS001"""", """"Pow"&amp;"er"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS002"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM30°"""", """"CCT"""""&amp;": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS003"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Stre"&amp;"ngth"""": """"IK10""""}
-{""""SKU"""":""""HRS004"""", """"Power"""": """"1.2W"""", """"Optics"""": """"SYM60°"""", """"CCT"""": """"4000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-{""""SKU"""":""""HRS005"""", """"Power"""&amp;""": """"1.2W"""", """"Optics"""": """"ASYM50°"""", """"CCT"""": """"3000K"""", """"IP Rating"""": """"IP67"""", """"Impact Strength"""": """"IK10""""}
-### Example Output:
-{
-  """"Options"""": {
-    """"Power"""": [
-      {""""name"""": """"1.2W"""", """""&amp;"id"""": """"101""""}
-    ],
-    """"Optics"""": [
-      {""""name"""": """"SYM30°"""", """"id"""": """"102""""},
-      {""""name"""": """"SYM60°"""", """"id"""": """"103""""},
-      {""""name"""": """"ASYM50°"""", """"id"""": """"104""""}
-    ],
-    """"C"&amp;"CT"""": [
-      {""""name"""": """"3000K"""", """"id"""": """"105""""},
-      {""""name"""": """"4000K"""", """"id"""": """"106""""}
-    ],
-    """"IP Rating"""": [
-      {""""name"""": """"IP67"""", """"id"""": """"107""""}
-    ],
-    """"Impact Strength"&amp;""""": [
-      {""""name"""": """"IK10"""", """"id"""": """"108""""}
-    ]
-  },
-  """"Constraints"""": {
-    """"104"""": [106]
-  },
-""""sku_mappings"""": [
-      { """"sku"""": """"HRS001"""", """"combination"""": [""""101"""", """"102"""", """"105"""", "&amp;"""""107"""", """"108""""] },
-      { """"sku"""": """"HRS002"""", """"combination"""": [""""101"""", """"102"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS003"""", """"combination"""": [""""101"""", """"103"""", """"105"""", "&amp;"""""107"""", """"108""""] },
-      { """"sku"""": """"HRS004"""", """"combination"""": [""""101"""", """"103"""", """"106"""", """"107"""", """"108""""] },
-      { """"sku"""": """"HRS005"""", """"combination"""": [""""101"""", """"104"""", """"105"""", "&amp;"""""107"""", """"108""""] },
-      { """"sku"""": """"HRS006"""", """"combination"""": [""""101"""", """"104"""", """"106"""", """"107"""", """"108""""] }
-    ]
-}
-Process the following product variant combinations and output the """"Options"""" and """"C"&amp;"onstraints"""" JSON:"", Q6)"),"{""Options"": {""Power"": [{""name"": ""7W"", ""id"": ""101""}], ""CCT"": [{""name"": ""6000K"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V"", ""id"": ""103""}], ""IP Rating"": [{""name"": ""IP68"", ""id"": ""104""}]}, ""Constraints"": {}, ""sku_ma"&amp;"ppings"": [{""sku"": ""PL002"", ""combination"": [""101"", ""102"", ""103"", ""104""]}]}")</f>
-        <v>{"Options": {"Power": [{"name": "7W", "id": "101"}], "CCT": [{"name": "6000K", "id": "102"}], "Voltage": [{"name": "12V", "id": "103"}], "IP Rating": [{"name": "IP68", "id": "104"}]}, "Constraints": {}, "sku_mappings": [{"sku": "PL002", "combination": ["101", "102", "103", "104"]}]}</v>
-      </c>
-      <c r="U6" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="V6" s="17" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract options object from the json"", U6)"),"{""Power"": [{""name"": ""7W"", ""id"": ""101""}], ""CCT"": [{""name"": ""6000K"", ""id"": ""102""}], ""Voltage"": [{""name"": ""12V"", ""id"": ""103""}], ""IP Rating"": [{""name"": ""IP68"", ""id"": ""104""}]}")</f>
-        <v>{"Power": [{"name": "7W", "id": "101"}], "CCT": [{"name": "6000K", "id": "102"}], "Voltage": [{"name": "12V", "id": "103"}], "IP Rating": [{"name": "IP68", "id": "104"}]}</v>
-      </c>
-      <c r="W6" s="17" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract constraints object from the json"", U6)"),"{}")</f>
-        <v>{}</v>
-      </c>
-      <c r="X6" s="17" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Extract sku_mappings object from the json"", U6)"),"[{""sku"": ""PL002"", ""combination"": [""101"", ""102"", ""103"", ""104""]}]")</f>
-        <v>[{"sku": "PL002", "combination": ["101", "102", "103", "104"]}]</v>
-      </c>
+      <c r="R6" s="11"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="11"/>
+      <c r="U6" s="16"/>
+      <c r="V6" s="17"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="17"/>
       <c r="Y6" s="15" t="s">
         <v>40</v>
       </c>
       <c r="Z6" s="15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AA6" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AB6" s="18"/>
       <c r="AC6" s="19" t="str">
@@ -1804,7 +1733,7 @@
         <v>pool light, 6000k, ip68 waterproof, 7w led, 12v lighting, aquatic light</v>
       </c>
       <c r="AD6" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7">

</xml_diff>